<commit_message>
Warn on any F3a declarations since people are still being surprised by the change
</commit_message>
<xml_diff>
--- a/tests/SENIOR-Team_Free-PRELIMS-OCC-.xlsx
+++ b/tests/SENIOR-Team_Free-PRELIMS-OCC-.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leahy\RustroverProjects\check_cards\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F622788-5378-4F4A-A02F-48369857F54E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA2CD7BB-2B46-4F34-91A5-8422C18E33C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{8987486B-5DC1-406A-92BD-FEEC5C92F2E7}"/>
   </bookViews>
@@ -234,9 +234,6 @@
     <t>Test</t>
   </si>
   <si>
-    <t xml:space="preserve"> FB F6a AB A6 S1 AB 2R1 F1a F2b F3a</t>
-  </si>
-  <si>
     <t xml:space="preserve"> C4 C4 C4 RD2 S1</t>
   </si>
   <si>
@@ -250,6 +247,9 @@
   </si>
   <si>
     <t>ISS Coach Card Version: 3.0.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> FB F6a AB A6 S1 AB 2R1 F1a F2b F3b</t>
   </si>
 </sst>
 </file>
@@ -434,6 +434,16 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
@@ -447,16 +457,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -804,96 +804,96 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="19"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="23"/>
     </row>
     <row r="2" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="16" t="s">
+      <c r="B2" s="18"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="15"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="19"/>
     </row>
     <row r="3" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="14"/>
-      <c r="C3" s="15"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="15"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="19"/>
     </row>
     <row r="4" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="14"/>
-      <c r="C4" s="15"/>
-      <c r="D4" s="16" t="s">
+      <c r="B4" s="18"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14"/>
-      <c r="H4" s="15"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="18"/>
+      <c r="G4" s="18"/>
+      <c r="H4" s="19"/>
     </row>
     <row r="5" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="23" t="s">
+      <c r="A5" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="23"/>
-      <c r="C5" s="23"/>
-      <c r="D5" s="16" t="s">
+      <c r="B5" s="16"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14"/>
-      <c r="H5" s="15"/>
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="19"/>
     </row>
     <row r="6" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="14"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="15"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="19"/>
     </row>
     <row r="7" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="14"/>
-      <c r="C7" s="15"/>
-      <c r="D7" s="16" t="s">
+      <c r="B7" s="18"/>
+      <c r="C7" s="19"/>
+      <c r="D7" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="15"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="19"/>
     </row>
     <row r="8" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
@@ -908,16 +908,16 @@
       <c r="H8" s="1"/>
     </row>
     <row r="9" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="20" t="s">
+      <c r="A9" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="21"/>
-      <c r="C9" s="21"/>
-      <c r="D9" s="21"/>
-      <c r="E9" s="21"/>
-      <c r="F9" s="21"/>
-      <c r="G9" s="21"/>
-      <c r="H9" s="22"/>
+      <c r="B9" s="14"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="15"/>
     </row>
     <row r="10" spans="1:8" ht="29.4" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
@@ -1011,7 +1011,7 @@
         <v>29</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F14" s="6"/>
       <c r="G14" s="8">
@@ -1085,7 +1085,7 @@
       </c>
       <c r="D18" s="7"/>
       <c r="E18" s="11" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>39</v>
@@ -1123,7 +1123,7 @@
       </c>
       <c r="D20" s="7"/>
       <c r="E20" s="12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>43</v>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="D22" s="7"/>
       <c r="E22" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>47</v>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="D24" s="7"/>
       <c r="E24" s="11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>39</v>
@@ -1393,7 +1393,7 @@
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
@@ -1615,6 +1615,13 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="D4:H4"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="D3:H3"/>
     <mergeCell ref="A9:H9"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A6:C6"/>
@@ -1622,13 +1629,6 @@
     <mergeCell ref="D6:H6"/>
     <mergeCell ref="A7:C7"/>
     <mergeCell ref="D7:H7"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="D4:H4"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="D3:H3"/>
   </mergeCells>
   <pageMargins left="6.9444444444444441E-3" right="6.9444444444444441E-3" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Use types instead of strings for declarations
This massivly reworks how the checker works. Now instead of strings
everywhere we have a huge amount of enums. This ends up being quite
a bit more code, but it should be much harder to make typos that
introduce false negatives.

With this, it is easy to calculate DDs for acros and hybrids, so
validation of that is added to the checker. As a bonus, this also
makes the DD checks not depend on ISS, so if you are using the
text-only version, the checker will now yell at you there if your
DD is too high.

Close #27
</commit_message>
<xml_diff>
--- a/tests/SENIOR-Team_Free-PRELIMS-OCC-.xlsx
+++ b/tests/SENIOR-Team_Free-PRELIMS-OCC-.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leahy\RustroverProjects\check_cards\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA2CD7BB-2B46-4F34-91A5-8422C18E33C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CD1FBC0-04E1-4942-BA54-8D392483C6DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{8987486B-5DC1-406A-92BD-FEEC5C92F2E7}"/>
   </bookViews>
@@ -246,10 +246,10 @@
     <t xml:space="preserve"> CB+ A5 1RB A6 CB+ CB+ A1c 2RB</t>
   </si>
   <si>
-    <t>ISS Coach Card Version: 3.0.5</t>
-  </si>
-  <si>
     <t xml:space="preserve"> FB F6a AB A6 S1 AB 2R1 F1a F2b F3b</t>
+  </si>
+  <si>
+    <t>ISS Coach Card Version: 3.0.6</t>
   </si>
 </sst>
 </file>
@@ -977,7 +977,7 @@
       </c>
       <c r="F12" s="6"/>
       <c r="G12" s="8">
-        <v>2.238</v>
+        <v>2.2250000000000001</v>
       </c>
       <c r="H12" s="10" t="s">
         <v>26</v>
@@ -1015,7 +1015,7 @@
       </c>
       <c r="F14" s="6"/>
       <c r="G14" s="8">
-        <v>1.875</v>
+        <v>2.125</v>
       </c>
       <c r="H14" s="10" t="s">
         <v>30</v>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="F16" s="6"/>
       <c r="G16" s="8">
-        <v>1.9</v>
+        <v>1.925</v>
       </c>
       <c r="H16" s="10" t="s">
         <v>35</v>
@@ -1085,13 +1085,13 @@
       </c>
       <c r="D18" s="7"/>
       <c r="E18" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>39</v>
       </c>
       <c r="G18" s="8">
-        <v>3.75</v>
+        <v>4.05</v>
       </c>
       <c r="H18" s="10" t="s">
         <v>40</v>
@@ -1205,7 +1205,7 @@
         <v>39</v>
       </c>
       <c r="G24" s="8">
-        <v>3.35</v>
+        <v>3.55</v>
       </c>
       <c r="H24" s="10" t="s">
         <v>51</v>
@@ -1393,7 +1393,7 @@
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>

</xml_diff>